<commit_message>
fix: demo loader works offline and via file:// protocol
Embeds cnt_demo.xlsx as base64 fallback so the demo button works when
opening cnt.html directly (file:// URLs block fetch). Tries fetch first
(server), falls back to embedded data. Also regenerated demo Excel with
tasaCreacion column and fixed writeEsencialesSheet range/headers.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cnt_demo.xlsx
+++ b/cnt_demo.xlsx
@@ -403,12 +403,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D8"/>
-  <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="45.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -510,21 +504,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L18"/>
-  <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="8.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="35.83203125" customWidth="1"/>
-    <col min="12" max="12" width="10.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:M18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -571,14 +551,17 @@
         <v xml:space="preserve">Original
 (USD)</v>
       </c>
-      <c r="J3" t="str" xml:space="preserve">
+      <c r="J3" t="str">
+        <v>TasaCreacion</v>
+      </c>
+      <c r="K3" t="str" xml:space="preserve">
         <v xml:space="preserve">Fecha
 Límite</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str">
         <v>Notas</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
         <v>Pagado_Mes</v>
       </c>
     </row>
@@ -610,13 +593,16 @@
       <c r="I4">
         <v>89430</v>
       </c>
-      <c r="J4" t="str">
+      <c r="J4">
+        <v>54.5</v>
+      </c>
+      <c r="K4" t="str">
         <v>2041-03-05</v>
       </c>
-      <c r="K4" t="str">
+      <c r="L4" t="str">
         <v>Banco BHD · cuota fija 15 años</v>
       </c>
-      <c r="L4" t="str">
+      <c r="M4" t="str">
         <v>SI</v>
       </c>
     </row>
@@ -649,12 +635,15 @@
         <v>0</v>
       </c>
       <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
         <v>—</v>
       </c>
-      <c r="K5" t="str">
+      <c r="L5" t="str">
         <v>Incluye agua y basura</v>
       </c>
-      <c r="L5" t="str">
+      <c r="M5" t="str">
         <v>SI</v>
       </c>
     </row>
@@ -686,13 +675,16 @@
       <c r="I6">
         <v>15447</v>
       </c>
-      <c r="J6" t="str">
+      <c r="J6">
+        <v>57.2</v>
+      </c>
+      <c r="K6" t="str">
         <v>2028-09-15</v>
       </c>
-      <c r="K6" t="str">
+      <c r="L6" t="str">
         <v>Banreservas · 5 años</v>
       </c>
-      <c r="L6" t="str">
+      <c r="M6" t="str">
         <v>NO</v>
       </c>
     </row>
@@ -725,12 +717,15 @@
         <v>0</v>
       </c>
       <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
         <v>—</v>
       </c>
-      <c r="K7" t="str">
+      <c r="L7" t="str">
         <v>Pago mínimo no cubre intereses</v>
       </c>
-      <c r="L7" t="str">
+      <c r="M7" t="str">
         <v>NO</v>
       </c>
     </row>
@@ -762,13 +757,16 @@
       <c r="I8">
         <v>0</v>
       </c>
-      <c r="J8" t="str">
+      <c r="J8">
+        <v>60.5</v>
+      </c>
+      <c r="K8" t="str">
         <v>—</v>
       </c>
-      <c r="K8" t="str">
+      <c r="L8" t="str">
         <v>Consolidar con Visa</v>
       </c>
-      <c r="L8" t="str">
+      <c r="M8" t="str">
         <v>NO</v>
       </c>
     </row>
@@ -801,12 +799,15 @@
         <v>0</v>
       </c>
       <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
         <v>—</v>
       </c>
-      <c r="K9" t="str">
+      <c r="L9" t="str">
         <v>Promedio últimos 3 meses</v>
       </c>
-      <c r="L9" t="str">
+      <c r="M9" t="str">
         <v>SI</v>
       </c>
     </row>
@@ -839,12 +840,15 @@
         <v>0</v>
       </c>
       <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
         <v>—</v>
       </c>
-      <c r="K10" t="str">
+      <c r="L10" t="str">
         <v>Internet 200Mbps + TV + tel</v>
       </c>
-      <c r="L10" t="str">
+      <c r="M10" t="str">
         <v>SI</v>
       </c>
     </row>
@@ -877,12 +881,15 @@
         <v>0</v>
       </c>
       <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
         <v>—</v>
       </c>
-      <c r="K11" t="str">
+      <c r="L11" t="str">
         <v>Plan familiar 3 líneas</v>
       </c>
-      <c r="L11" t="str">
+      <c r="M11" t="str">
         <v>SI</v>
       </c>
     </row>
@@ -915,12 +922,15 @@
         <v>0</v>
       </c>
       <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
         <v>—</v>
       </c>
-      <c r="K12" t="str">
+      <c r="L12" t="str">
         <v>Plan familiar complementario</v>
       </c>
-      <c r="L12" t="str">
+      <c r="M12" t="str">
         <v>SI</v>
       </c>
     </row>
@@ -953,12 +963,15 @@
         <v>0</v>
       </c>
       <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
         <v>—</v>
       </c>
-      <c r="K13" t="str">
+      <c r="L13" t="str">
         <v>Estimado semanal ~RD$5,500</v>
       </c>
-      <c r="L13" t="str">
+      <c r="M13" t="str">
         <v>NO</v>
       </c>
     </row>
@@ -991,12 +1004,15 @@
         <v>0</v>
       </c>
       <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
         <v>—</v>
       </c>
-      <c r="K14" t="str">
+      <c r="L14" t="str">
         <v>~3 tanques al mes</v>
       </c>
-      <c r="L14" t="str">
+      <c r="M14" t="str">
         <v>NO</v>
       </c>
     </row>
@@ -1029,12 +1045,15 @@
         <v>0</v>
       </c>
       <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
         <v>—</v>
       </c>
-      <c r="K15" t="str">
+      <c r="L15" t="str">
         <v>Membresía mensual</v>
       </c>
-      <c r="L15" t="str">
+      <c r="M15" t="str">
         <v>SI</v>
       </c>
     </row>
@@ -1067,12 +1086,15 @@
         <v>0</v>
       </c>
       <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
         <v>—</v>
       </c>
-      <c r="K16" t="str">
+      <c r="L16" t="str">
         <v>Plan estándar ambos</v>
       </c>
-      <c r="L16" t="str">
+      <c r="M16" t="str">
         <v>SI</v>
       </c>
     </row>
@@ -1105,12 +1127,15 @@
         <v>0</v>
       </c>
       <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
         <v>—</v>
       </c>
-      <c r="K17" t="str">
+      <c r="L17" t="str">
         <v>Curso trimestral · cuota mensual</v>
       </c>
-      <c r="L17" t="str">
+      <c r="M17" t="str">
         <v>SI</v>
       </c>
     </row>
@@ -1143,18 +1168,21 @@
         <v>0</v>
       </c>
       <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
         <v>—</v>
       </c>
-      <c r="K18" t="str">
+      <c r="L18" t="str">
         <v>Transferencia mensual fija</v>
       </c>
-      <c r="L18" t="str">
+      <c r="M18" t="str">
         <v>NO</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M18"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1162,12 +1190,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D9"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1263,13 +1285,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E17"/>
-  <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1484,19 +1499,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K21"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="6.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="8.83203125" customWidth="1"/>
-    <col min="11" max="11" width="45.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2191,12 +2193,6 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D6"/>
-  <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>